<commit_message>
Sync PLOS revision tables and source audit documentation
</commit_message>
<xml_diff>
--- a/PONE_D_26_35909/supporting_data/S10_Data.xlsx
+++ b/PONE_D_26_35909/supporting_data/S10_Data.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TableS8b_parameter_sensitivity_" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TableS10a_exact_meta_calibratio" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TableS10b_exact_meta_null_tail" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TableS10a_omissions" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TableS7a_uniform_annotation_pat'!$A$1:$I$29</definedName>
@@ -22,6 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TableS8b_parameter_sensitivity_'!$A$1:$I$188</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'TableS10a_exact_meta_calibratio'!$A$1:$N$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'TableS10b_exact_meta_null_tail'!$A$1:$E$243</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'TableS10a_omissions'!$A$1:$F$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -30,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,8 +43,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +58,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002D7F82"/>
       </patternFill>
     </fill>
   </fills>
@@ -67,12 +78,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -485,7 +497,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -684,6 +695,62 @@
       </c>
       <c r="F11" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Long-table conversion</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>JSON fields are expanded into linked worksheets; source_excel_row and record_index preserve the original ordering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Numeric precision</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Numbers formerly embedded in JSON are stored as exact decimal text to preserve every supplied digit. No values or statistical results were recalculated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Patient keys</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Patient codes are sequential within cohort. Each patient table has one row per patient per ligand or regional comparison.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TableS10a_omissions</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TableS10a_exact_meta_calibratio</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>exact_loo_results</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -9668,7 +9735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9740,20 +9807,15 @@
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>exact_loo_results</t>
+          <t>full_signflip_patterns</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>full_signflip_patterns</t>
+          <t>exact_signflip_q_value</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>exact_signflip_q_value</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>exact_loo_q_value</t>
         </is>
@@ -9792,18 +9854,13 @@
       <c r="J2" t="n">
         <v>0.000244140625</v>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>[{"omitted": "GSE211376", "meta_z": 3.062002587210068, "exact_p_value": 0.0001220703125}, {"omitted": "GSE273274", "meta_z": 3.5750709135967043, "exact_p_value": 1.52587890625e-05}, {"omitted": "GSE274987", "meta_z": 2.8668566448234234, "exact_p_value": 0.000244140625}, {"omitted": "GSE286419", "meta_z": 3.4161543700985426, "exact_p_value": 3.0517578125e-05}]</t>
-        </is>
+      <c r="K2" t="n">
+        <v>1048576</v>
       </c>
       <c r="L2" t="n">
-        <v>1048576</v>
+        <v>1.1444091796875e-05</v>
       </c>
       <c r="M2" t="n">
-        <v>1.1444091796875e-05</v>
-      </c>
-      <c r="N2" t="n">
         <v>0.00146484375</v>
       </c>
     </row>
@@ -9840,18 +9897,13 @@
       <c r="J3" t="n">
         <v>0.005859375</v>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>[{"omitted": "GSE211376", "meta_z": 3.062002587210068, "exact_p_value": 0.0001220703125}, {"omitted": "GSE273274", "meta_z": 3.02612364906194, "exact_p_value": 0.0004119873046875}, {"omitted": "GSE274987", "meta_z": 2.239111431498328, "exact_p_value": 0.005859375}, {"omitted": "GSE286419", "meta_z": 2.8503124814558642, "exact_p_value": 0.000823974609375}]</t>
-        </is>
+      <c r="K3" t="n">
+        <v>1048576</v>
       </c>
       <c r="L3" t="n">
-        <v>1048576</v>
+        <v>0.0002346038818359</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0002346038818359</v>
-      </c>
-      <c r="N3" t="n">
         <v>0.017578125</v>
       </c>
     </row>
@@ -9888,18 +9940,13 @@
       <c r="J4" t="n">
         <v>0.041015625</v>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>[{"omitted": "GSE211376", "meta_z": 2.355064183534596, "exact_p_value": 0.0042724609375}, {"omitted": "GSE273274", "meta_z": 1.997998296565367, "exact_p_value": 0.023345947265625}, {"omitted": "GSE274987", "meta_z": 1.7970297627507015, "exact_p_value": 0.027587890625}, {"omitted": "GSE286419", "meta_z": 1.7905451252761742, "exact_p_value": 0.041015625}]</t>
-        </is>
+      <c r="K4" t="n">
+        <v>1048576</v>
       </c>
       <c r="L4" t="n">
-        <v>1048576</v>
+        <v>0.0142097473144531</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0142097473144531</v>
-      </c>
-      <c r="N4" t="n">
         <v>0.08203125</v>
       </c>
     </row>
@@ -9936,18 +9983,13 @@
       <c r="J5" t="n">
         <v>0.796875</v>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>[{"omitted": "GSE211376", "meta_z": 2.4120318065602153, "exact_p_value": 0.003173828125}, {"omitted": "GSE273274", "meta_z": 0.599012170518534, "exact_p_value": 0.488525390625}, {"omitted": "GSE274987", "meta_z": -0.2207667706508716, "exact_p_value": 0.796875}, {"omitted": "GSE286419", "meta_z": 0.6719902263268205, "exact_p_value": 0.42681884765625}]</t>
-        </is>
+      <c r="K5" t="n">
+        <v>1048576</v>
       </c>
       <c r="L5" t="n">
-        <v>1048576</v>
+        <v>0.3558826446533203</v>
       </c>
       <c r="M5" t="n">
-        <v>0.3558826446533203</v>
-      </c>
-      <c r="N5" t="n">
         <v>0.851593017578125</v>
       </c>
     </row>
@@ -9984,18 +10026,13 @@
       <c r="J6" t="n">
         <v>0.851593017578125</v>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>[{"omitted": "GSE211376", "meta_z": 0.7279665087583541, "exact_p_value": 0.3892822265625}, {"omitted": "GSE273274", "meta_z": 1.033446297146116, "exact_p_value": 0.2382354736328125}, {"omitted": "GSE274987", "meta_z": 0.9711826743099569, "exact_p_value": 0.23583984375}, {"omitted": "GSE286419", "meta_z": 0.1602168962885174, "exact_p_value": 0.851593017578125}]</t>
-        </is>
+      <c r="K6" t="n">
+        <v>1048576</v>
       </c>
       <c r="L6" t="n">
-        <v>1048576</v>
+        <v>0.3988929748535156</v>
       </c>
       <c r="M6" t="n">
-        <v>0.3988929748535156</v>
-      </c>
-      <c r="N6" t="n">
         <v>0.851593017578125</v>
       </c>
     </row>
@@ -10032,18 +10069,13 @@
       <c r="J7" t="n">
         <v>0.442138671875</v>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>[{"omitted": "GSE211376", "meta_z": 1.1737362735217778, "exact_p_value": 0.1651611328125}, {"omitted": "GSE273274", "meta_z": 0.8549478462454171, "exact_p_value": 0.332061767578125}, {"omitted": "GSE274987", "meta_z": -0.6337724950991952, "exact_p_value": 0.442138671875}, {"omitted": "GSE286419", "meta_z": 0.8219405190016984, "exact_p_value": 0.34295654296875}]</t>
-        </is>
+      <c r="K7" t="n">
+        <v>1048576</v>
       </c>
       <c r="L7" t="n">
-        <v>1048576</v>
+        <v>0.4365158081054687</v>
       </c>
       <c r="M7" t="n">
-        <v>0.4365158081054687</v>
-      </c>
-      <c r="N7" t="n">
         <v>0.6632080078125</v>
       </c>
     </row>
@@ -14698,4 +14730,731 @@
   <autoFilter ref="A1:E243"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>source_excel_row</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>record_index</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>gene</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>omitted</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>meta_z</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>exact_p_value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TGFB2</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>GSE211376</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>3.062002587210068</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.0001220703125</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TGFB2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>GSE273274</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>3.5750709135967043</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1.52587890625e-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TGFB2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>GSE274987</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2.8668566448234234</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.000244140625</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TGFB2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>GSE286419</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>3.4161543700985426</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>3.0517578125e-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CSF1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>GSE211376</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>3.062002587210068</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.0001220703125</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CSF1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>GSE273274</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>3.02612364906194</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.0004119873046875</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CSF1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>GSE274987</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2.239111431498328</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.005859375</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CSF1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>GSE286419</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2.8503124814558642</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.000823974609375</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ANXA1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>GSE211376</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2.355064183534596</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.0042724609375</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ANXA1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>GSE273274</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.997998296565367</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.023345947265625</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ANXA1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>GSE274987</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1.7970297627507015</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.027587890625</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ANXA1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>GSE286419</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.7905451252761742</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0.041015625</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CCL2</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>GSE211376</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2.4120318065602153</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0.003173828125</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CCL2</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>GSE273274</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0.599012170518534</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0.488525390625</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CCL2</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>GSE274987</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>-0.2207667706508716</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.796875</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>5</v>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CCL2</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>GSE286419</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0.6719902263268205</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.42681884765625</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TGFB1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>GSE211376</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0.7279665087583541</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.3892822265625</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>6</v>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TGFB1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>GSE273274</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.033446297146116</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0.2382354736328125</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>6</v>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>TGFB1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>GSE274987</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0.9711826743099569</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>0.23583984375</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>6</v>
+      </c>
+      <c r="B21" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>TGFB1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>GSE286419</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>0.1602168962885174</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>0.851593017578125</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>7</v>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SPP1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>GSE211376</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1.1737362735217778</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>0.1651611328125</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>7</v>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>SPP1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>GSE273274</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>0.8549478462454171</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0.332061767578125</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>SPP1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>GSE274987</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>-0.6337724950991952</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>0.442138671875</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>SPP1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>GSE286419</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>0.8219405190016984</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>0.34295654296875</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F25"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>